<commit_message>
Daily EOD data and reports for 2026-09-28
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260928.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260928.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.87</v>
+        <v>1.865</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.03</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.32%</t>
+          <t>-1.58%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>286448.47</v>
+        <v>285682.57</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-3829.52</v>
+        <v>-4595.43</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.585</v>
+        <v>2.59</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.02</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.96%</t>
+          <t>-0.77%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>180950</v>
+        <v>181300</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-1750</v>
+        <v>-1400</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>59.98</v>
+        <v>59.8</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.74</v>
+        <v>-0.92</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-1.22%</t>
+          <t>-1.52%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>479840</v>
+        <v>478400</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-5920</v>
+        <v>-7360</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>151.925</v>
+        <v>151.52</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1.095</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.73%</t>
+          <t>0.46%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.905</v>
+        <v>0.89</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.02</v>
+        <v>-0.035</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-2.16%</t>
+          <t>-3.78%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>9050</v>
+        <v>8900</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>-200</v>
+        <v>-350</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>180.595</v>
+        <v>181.91</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.645</v>
+        <v>4.96</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.06%</t>
+          <t>2.80%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>722380</v>
+        <v>727640</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>14580</v>
+        <v>19840</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>15.91</v>
+        <v>16.02</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.29</v>
+        <v>-0.18</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-1.11%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>48445.95</v>
+        <v>48780.9</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-883.05</v>
+        <v>-548.1</v>
       </c>
     </row>
     <row r="13">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.98</v>
+        <v>35.04</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.49</v>
+        <v>0.55</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.42%</t>
+          <t>1.59%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.94</v>
+        <v>31.77</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.22</v>
+        <v>0.05</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.69%</t>
+          <t>0.16%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41138.72</v>
+        <v>40919.76</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>283.36</v>
+        <v>64.40000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1774488.91</v>
+        <v>1777858.99</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>847.37</v>
+        <v>4217.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>